<commit_message>
Added up-to-date raw data of data articles analysis; Added a template at the head of index.qmd for authors details; Rendered index as html.
</commit_message>
<xml_diff>
--- a/data/raw/data_articles/datajournal_articles git V final_1.xlsx
+++ b/data/raw/data_articles/datajournal_articles git V final_1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29816"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bliv10\Desktop\DCC github\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AVIHAY\git\DCC-v3\data\raw\data_articles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{EF7AA90C-37E4-49C0-8C4B-1A935935D77E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9A0BBA8-6B7D-4422-BDA7-52776CA9A06F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D91033A-900E-4576-8819-277B4CECD31A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="16800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="10440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="datajournal_articles - analysis" sheetId="1" r:id="rId1"/>
@@ -31,6 +31,9 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -41,10 +44,10 @@
     <t>Number</t>
   </si>
   <si>
-    <t>date of check</t>
-  </si>
-  <si>
-    <t>doi</t>
+    <t>Date of check</t>
+  </si>
+  <si>
+    <t>Data Article DOI</t>
   </si>
   <si>
     <t>pmid</t>
@@ -594,7 +597,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1080,54 +1083,59 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="43">
-    <cellStyle name="20 % - Akzent1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20 % - Akzent2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20 % - Akzent3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20 % - Akzent4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20 % - Akzent5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20 % - Akzent6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40 % - Akzent1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40 % - Akzent2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40 % - Akzent3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40 % - Akzent4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40 % - Akzent5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40 % - Akzent6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60 % - Akzent1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60 % - Akzent2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60 % - Akzent3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60 % - Akzent4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60 % - Akzent5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60 % - Akzent6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Akzent1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Akzent2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Akzent3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Akzent4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Akzent5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Akzent6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Ausgabe" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Berechnung" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Eingabe" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Ergebnis" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Erklärender Text" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Gut" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
     <cellStyle name="Hyperlink" xfId="42" xr:uid="{00000000-000B-0000-0000-000008000000}"/>
+    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
-    <cellStyle name="Notiz" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Schlecht" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
-    <cellStyle name="Überschrift" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Überschrift 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Überschrift 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Überschrift 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Überschrift 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Verknüpfte Zelle" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Warnender Text" xfId="14" builtinId="11" customBuiltin="1"/>
-    <cellStyle name="Zelle überprüfen" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1143,9 +1151,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1183,7 +1191,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1289,7 +1297,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1431,7 +1439,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1440,19 +1448,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AK23"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.28515625" customWidth="1"/>
-    <col min="2" max="2" width="13.7109375" customWidth="1"/>
+    <col min="1" max="1" width="9.85546875" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="28.85546875" customWidth="1"/>
     <col min="5" max="5" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
@@ -1561,11 +1569,11 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:37" ht="70.5" customHeight="1">
+    <row r="2" spans="1:37" ht="70.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>37</v>
       </c>
       <c r="C2" t="s">
@@ -1674,11 +1682,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:37">
+    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="2">
         <v>45574</v>
       </c>
       <c r="C3" t="s">
@@ -1787,11 +1795,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:37">
+    <row r="4" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="2">
         <v>45605</v>
       </c>
       <c r="C4" t="s">
@@ -1900,11 +1908,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:37">
+    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="2">
         <v>45629</v>
       </c>
       <c r="C5" t="s">
@@ -2013,11 +2021,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:37">
+    <row r="6" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="2">
         <v>45629</v>
       </c>
       <c r="C6" t="s">
@@ -2126,11 +2134,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:37">
+    <row r="7" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="2" t="s">
         <v>83</v>
       </c>
       <c r="C7" t="s">
@@ -2239,11 +2247,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:37">
+    <row r="8" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="2" t="s">
         <v>91</v>
       </c>
       <c r="C8" t="s">
@@ -2352,11 +2360,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:37">
+    <row r="9" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" s="1">
+      <c r="B9" s="2">
         <v>45719</v>
       </c>
       <c r="C9" t="s">
@@ -2465,11 +2473,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:37">
+    <row r="10" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10" s="1">
+      <c r="B10" s="2">
         <v>45629</v>
       </c>
       <c r="C10" t="s">
@@ -2578,11 +2586,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:37" ht="15">
+    <row r="11" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11" s="1">
+      <c r="B11" s="2">
         <v>45629</v>
       </c>
       <c r="C11" t="s">
@@ -2691,11 +2699,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:37">
+    <row r="12" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="2" t="s">
         <v>113</v>
       </c>
       <c r="C12" t="s">
@@ -2804,11 +2812,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:37">
+    <row r="13" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="2" t="s">
         <v>113</v>
       </c>
       <c r="C13" t="s">
@@ -2917,11 +2925,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:37">
+    <row r="14" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="2" t="s">
         <v>113</v>
       </c>
       <c r="C14" t="s">
@@ -3030,11 +3038,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:37">
+    <row r="15" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="2" t="s">
         <v>113</v>
       </c>
       <c r="C15" t="s">
@@ -3143,11 +3151,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:37">
+    <row r="16" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="2" t="s">
         <v>113</v>
       </c>
       <c r="C16" t="s">
@@ -3256,11 +3264,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:37">
+    <row r="17" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
-      <c r="B17" s="1">
+      <c r="B17" s="2">
         <v>45629</v>
       </c>
       <c r="C17" t="s">
@@ -3369,11 +3377,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:37">
+    <row r="18" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
-      <c r="B18" s="1">
+      <c r="B18" s="2">
         <v>45629</v>
       </c>
       <c r="C18" t="s">
@@ -3482,11 +3490,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:37">
+    <row r="19" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="2" t="s">
         <v>91</v>
       </c>
       <c r="C19" t="s">
@@ -3595,11 +3603,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:37">
+    <row r="20" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="2" t="s">
         <v>91</v>
       </c>
       <c r="C20" t="s">
@@ -3708,11 +3716,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:37">
+    <row r="21" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
-      <c r="B21" s="1">
+      <c r="B21" s="2">
         <v>45629</v>
       </c>
       <c r="C21" t="s">
@@ -3821,11 +3829,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:37">
+    <row r="22" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
-      <c r="B22" s="1">
+      <c r="B22" s="2">
         <v>45629</v>
       </c>
       <c r="C22" t="s">
@@ -3934,11 +3942,11 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:37">
+    <row r="23" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
-      <c r="B23" s="1">
+      <c r="B23" s="2">
         <v>45635</v>
       </c>
       <c r="C23" t="s">
@@ -4053,14 +4061,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a0e84d40-090a-490d-8a02-2942ffba970a" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="aaacefca-f467-416c-abd0-2b181dff1e20">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4259,22 +4265,50 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a0e84d40-090a-490d-8a02-2942ffba970a" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="aaacefca-f467-416c-abd0-2b181dff1e20">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C2D3F5D9-F66A-401E-BC58-4588B5177296}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{647AA23E-A486-48B9-BA40-113933E28953}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9691CDE3-47DE-4336-B4B1-23B29CAB7B59}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FE800AB4-95A0-4642-AA3E-75920632EF08}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="aaacefca-f467-416c-abd0-2b181dff1e20"/>
+    <ds:schemaRef ds:uri="a0e84d40-090a-490d-8a02-2942ffba970a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{647AA23E-A486-48B9-BA40-113933E28953}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C2D3F5D9-F66A-401E-BC58-4588B5177296}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a0e84d40-090a-490d-8a02-2942ffba970a"/>
+    <ds:schemaRef ds:uri="aaacefca-f467-416c-abd0-2b181dff1e20"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>